<commit_message>
added LCSC part numbers to JLC_BOM
</commit_message>
<xml_diff>
--- a/Altium_project/Project Outputs for UZ_D_Temperature_Card_LTC2983/Rev03/BOM_JLC/BOM_JLC_UZ_D_Temperature_Card_LTC2983_All_Thermocouple_Rev03.xlsx
+++ b/Altium_project/Project Outputs for UZ_D_Temperature_Card_LTC2983/Rev03/BOM_JLC/BOM_JLC_UZ_D_Temperature_Card_LTC2983_All_Thermocouple_Rev03.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20405"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projekte\UltraZohm\Work_Altium\uz_d_temperature\Altium_project\Project Outputs for UZ_D_Temperature_Card_LTC2983\Rev03\BOM_JLC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\UltraZohm\pcb_design\uz_d_temperature\Altium_project\Project Outputs for UZ_D_Temperature_Card_LTC2983\Rev03\BOM_JLC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1AF8AEBF-3696-4AE7-A071-C9F971377B25}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55D50CD7-CFC8-41B5-BA0B-081BB7A8EB2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="10215" xr2:uid="{EA51FFA7-EFCD-45C1-B18E-D554908E7AF3}"/>
+    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{EA51FFA7-EFCD-45C1-B18E-D554908E7AF3}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_JLC_UZ_D_Temperature_Card_L" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="66">
   <si>
     <t>Comment</t>
   </si>
@@ -102,9 +102,6 @@
     <t>R3A, R3B, R3C, R4A, R4B, R4C, R5A, R5B, R5C, R6A, R6B, R6C, R7A, R7B, R7C, R48, R50, R51, R52, R53, R54, R56, R57, R58, R59, R60, R62, R63, R64, R65, R66, R68, R70</t>
   </si>
   <si>
-    <t>[NoParam], C21189</t>
-  </si>
-  <si>
     <t>1k</t>
   </si>
   <si>
@@ -193,6 +190,42 @@
   </si>
   <si>
     <t>IPL1-115-01-XX-D-RA</t>
+  </si>
+  <si>
+    <t>C2803384</t>
+  </si>
+  <si>
+    <t>C5240381</t>
+  </si>
+  <si>
+    <t>C72043</t>
+  </si>
+  <si>
+    <t>C720204</t>
+  </si>
+  <si>
+    <t>C25804</t>
+  </si>
+  <si>
+    <t>C23228</t>
+  </si>
+  <si>
+    <t>C21189</t>
+  </si>
+  <si>
+    <t>C660948</t>
+  </si>
+  <si>
+    <t>C970824</t>
+  </si>
+  <si>
+    <t>C683919</t>
+  </si>
+  <si>
+    <t>C2684906</t>
+  </si>
+  <si>
+    <t>C7423882</t>
   </si>
 </sst>
 </file>
@@ -570,15 +603,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09CC2C1E-E235-439D-9A08-254F7C5B7961}">
   <dimension ref="A1:D19"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.28515625" customWidth="1"/>
-    <col min="2" max="2" width="17.85546875" customWidth="1"/>
-    <col min="3" max="3" width="24.7109375" customWidth="1"/>
-    <col min="4" max="4" width="16.7109375" customWidth="1"/>
+    <col min="1" max="1" width="19.26953125" customWidth="1"/>
+    <col min="2" max="2" width="17.81640625" customWidth="1"/>
+    <col min="3" max="3" width="24.7265625" customWidth="1"/>
+    <col min="4" max="4" width="16.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -592,7 +625,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -602,9 +635,11 @@
       <c r="C2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="1"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D2" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>7</v>
       </c>
@@ -614,9 +649,11 @@
       <c r="C3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="1"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D3" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
@@ -628,7 +665,7 @@
       </c>
       <c r="D4" s="1"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
@@ -638,9 +675,11 @@
       <c r="C5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="1"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D5" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>14</v>
       </c>
@@ -650,9 +689,11 @@
       <c r="C6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="1"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D6" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>17</v>
       </c>
@@ -662,9 +703,11 @@
       <c r="C7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="1"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D7" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -674,9 +717,11 @@
       <c r="C8" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="1"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D8" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>22</v>
       </c>
@@ -686,137 +731,149 @@
       <c r="C9" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="2" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
+      <c r="B10" s="2" t="s">
         <v>25</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>26</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
+      <c r="B11" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="C11" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="D11" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D11" s="1"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
+      <c r="B12" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>32</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>19</v>
       </c>
       <c r="D12" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
+      <c r="B13" s="2" t="s">
         <v>34</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>35</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>19</v>
       </c>
       <c r="D13" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" s="2" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
+      <c r="B14" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="C14" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="D14" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D14" s="2" t="s">
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" s="2" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
+      <c r="B15" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="C15" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="D15" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="D15" s="1"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
+      <c r="B16" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="C16" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="D16" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="D16" s="1"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
+      <c r="B17" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="C17" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="D17" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="D17" s="1"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
+      <c r="B18" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="C18" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C18" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D18" s="1"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
+      <c r="B19" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="C19" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="D19" s="1"/>
+      <c r="D19" s="1" t="s">
+        <v>65</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
maße minimal angepasst, runde ecken waren leicht verschoben
gerber files neu generiert und die alten gelöscht.
jlc nummern angepasst
</commit_message>
<xml_diff>
--- a/Altium_project/Project Outputs for UZ_D_Temperature_Card_LTC2983/Rev03/BOM_JLC/BOM_JLC_UZ_D_Temperature_Card_LTC2983_All_Thermocouple_Rev03.xlsx
+++ b/Altium_project/Project Outputs for UZ_D_Temperature_Card_LTC2983/Rev03/BOM_JLC/BOM_JLC_UZ_D_Temperature_Card_LTC2983_All_Thermocouple_Rev03.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20405"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\UltraZohm\pcb_design\uz_d_temperature\Altium_project\Project Outputs for UZ_D_Temperature_Card_LTC2983\Rev03\BOM_JLC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ga92wum\git\UltraZohm\PCB\UZ_D_Temperature\Altium_project\Project Outputs for UZ_D_Temperature_Card_LTC2983\Rev03\BOM_JLC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55D50CD7-CFC8-41B5-BA0B-081BB7A8EB2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F800283-30D7-4222-9EAD-A4D8EC828C11}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{EA51FFA7-EFCD-45C1-B18E-D554908E7AF3}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="69">
   <si>
     <t>Comment</t>
   </si>
@@ -168,9 +168,6 @@
     <t>SIP4DCDC</t>
   </si>
   <si>
-    <t>LTC2983</t>
-  </si>
-  <si>
     <t>U4A, U4B, U4C</t>
   </si>
   <si>
@@ -219,13 +216,25 @@
     <t>C970824</t>
   </si>
   <si>
-    <t>C683919</t>
-  </si>
-  <si>
     <t>C2684906</t>
   </si>
   <si>
     <t>C7423882</t>
+  </si>
+  <si>
+    <t>C427448</t>
+  </si>
+  <si>
+    <t>LTC2983ILX</t>
+  </si>
+  <si>
+    <t>C14663</t>
+  </si>
+  <si>
+    <t>Alternative</t>
+  </si>
+  <si>
+    <t>C7500913</t>
   </si>
 </sst>
 </file>
@@ -602,7 +611,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09CC2C1E-E235-439D-9A08-254F7C5B7961}">
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="19.26953125" customWidth="1"/>
@@ -611,7 +620,7 @@
     <col min="4" max="4" width="16.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -624,8 +633,11 @@
       <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E1" s="4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -636,10 +648,10 @@
         <v>6</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>7</v>
       </c>
@@ -650,10 +662,10 @@
         <v>6</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
@@ -663,9 +675,11 @@
       <c r="C4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="1"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D4" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
@@ -676,10 +690,10 @@
         <v>13</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>14</v>
       </c>
@@ -690,10 +704,10 @@
         <v>16</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>17</v>
       </c>
@@ -704,10 +718,10 @@
         <v>19</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -718,10 +732,10 @@
         <v>19</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>22</v>
       </c>
@@ -732,10 +746,10 @@
         <v>19</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>24</v>
       </c>
@@ -749,7 +763,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>27</v>
       </c>
@@ -760,10 +774,10 @@
         <v>29</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>30</v>
       </c>
@@ -777,7 +791,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>33</v>
       </c>
@@ -791,7 +805,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>36</v>
       </c>
@@ -805,7 +819,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>40</v>
       </c>
@@ -816,10 +830,10 @@
         <v>42</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>43</v>
       </c>
@@ -830,49 +844,52 @@
         <v>45</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="C17" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="D17" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="D17" s="1" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A18" s="2" t="s">
+      <c r="B18" s="2" t="s">
         <v>49</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>50</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="D18" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D18" t="s">
+        <v>68</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="C19" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>53</v>
-      </c>
       <c r="D19" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add solder bumper instead of pull-up at EEPROM write access protection pin
</commit_message>
<xml_diff>
--- a/Altium_project/Project Outputs for UZ_D_Temperature_Card_LTC2983/Rev03/BOM_JLC/BOM_JLC_UZ_D_Temperature_Card_LTC2983_All_Thermocouple_Rev03.xlsx
+++ b/Altium_project/Project Outputs for UZ_D_Temperature_Card_LTC2983/Rev03/BOM_JLC/BOM_JLC_UZ_D_Temperature_Card_LTC2983_All_Thermocouple_Rev03.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ga92wum\git\UltraZohm\PCB\UZ_D_Temperature\Altium_project\Project Outputs for UZ_D_Temperature_Card_LTC2983\Rev03\BOM_JLC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projekte\UltraZohm\Work_Altium\uz_d_temperature\Altium_project\Project Outputs for UZ_D_Temperature_Card_LTC2983\Rev03\BOM_JLC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F800283-30D7-4222-9EAD-A4D8EC828C11}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{60AA517B-9978-475A-94A9-61975E874F01}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{EA51FFA7-EFCD-45C1-B18E-D554908E7AF3}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="10215" xr2:uid="{4860BE7A-7AF4-4976-A364-F716E6499B9B}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_JLC_UZ_D_Temperature_Card_L" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="55">
   <si>
     <t>Comment</t>
   </si>
@@ -102,6 +102,9 @@
     <t>R3A, R3B, R3C, R4A, R4B, R4C, R5A, R5B, R5C, R6A, R6B, R6C, R7A, R7B, R7C, R48, R50, R51, R52, R53, R54, R56, R57, R58, R59, R60, R62, R63, R64, R65, R66, R68, R70</t>
   </si>
   <si>
+    <t>[NoParam], C21189</t>
+  </si>
+  <si>
     <t>1k</t>
   </si>
   <si>
@@ -123,7 +126,7 @@
     <t>4k7</t>
   </si>
   <si>
-    <t>R72, R73</t>
+    <t>R71, R72, R73</t>
   </si>
   <si>
     <t>C23162</t>
@@ -168,6 +171,9 @@
     <t>SIP4DCDC</t>
   </si>
   <si>
+    <t>LTC2983</t>
+  </si>
+  <si>
     <t>U4A, U4B, U4C</t>
   </si>
   <si>
@@ -187,54 +193,6 @@
   </si>
   <si>
     <t>IPL1-115-01-XX-D-RA</t>
-  </si>
-  <si>
-    <t>C2803384</t>
-  </si>
-  <si>
-    <t>C5240381</t>
-  </si>
-  <si>
-    <t>C72043</t>
-  </si>
-  <si>
-    <t>C720204</t>
-  </si>
-  <si>
-    <t>C25804</t>
-  </si>
-  <si>
-    <t>C23228</t>
-  </si>
-  <si>
-    <t>C21189</t>
-  </si>
-  <si>
-    <t>C660948</t>
-  </si>
-  <si>
-    <t>C970824</t>
-  </si>
-  <si>
-    <t>C2684906</t>
-  </si>
-  <si>
-    <t>C7423882</t>
-  </si>
-  <si>
-    <t>C427448</t>
-  </si>
-  <si>
-    <t>LTC2983ILX</t>
-  </si>
-  <si>
-    <t>C14663</t>
-  </si>
-  <si>
-    <t>Alternative</t>
-  </si>
-  <si>
-    <t>C7500913</t>
   </si>
 </sst>
 </file>
@@ -610,17 +568,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09CC2C1E-E235-439D-9A08-254F7C5B7961}">
-  <dimension ref="A1:E19"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05371DEE-CF93-4DE9-9C2F-732CEF61DEF1}">
+  <dimension ref="A1:D19"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.26953125" customWidth="1"/>
-    <col min="2" max="2" width="17.81640625" customWidth="1"/>
-    <col min="3" max="3" width="24.7265625" customWidth="1"/>
-    <col min="4" max="4" width="16.7265625" customWidth="1"/>
+    <col min="1" max="1" width="19.28515625" customWidth="1"/>
+    <col min="2" max="2" width="17.85546875" customWidth="1"/>
+    <col min="3" max="3" width="24.7109375" customWidth="1"/>
+    <col min="4" max="4" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -633,11 +591,8 @@
       <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -647,11 +602,9 @@
       <c r="C2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D2" s="1"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>7</v>
       </c>
@@ -661,11 +614,9 @@
       <c r="C3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D3" s="1"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
@@ -675,11 +626,9 @@
       <c r="C4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D4" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D4" s="1"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
@@ -689,11 +638,9 @@
       <c r="C5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D5" s="1"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>14</v>
       </c>
@@ -703,11 +650,9 @@
       <c r="C6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D6" s="1"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>17</v>
       </c>
@@ -717,11 +662,9 @@
       <c r="C7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D7" s="1"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -731,11 +674,9 @@
       <c r="C8" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D8" s="1"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>22</v>
       </c>
@@ -745,152 +686,137 @@
       <c r="C9" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D9" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D10" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D10" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+        <v>30</v>
+      </c>
+      <c r="D11" s="1"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>19</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>19</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+        <v>43</v>
+      </c>
+      <c r="D15" s="1"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+        <v>46</v>
+      </c>
+      <c r="D16" s="1"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>65</v>
+        <v>47</v>
       </c>
       <c r="B17" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D17" s="1"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C17" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="D17" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A18" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="D18" t="s">
-        <v>68</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D18" s="1"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>63</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="D19" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>